<commit_message>
v5.4: adopt Neon-only database architecture
</commit_message>
<xml_diff>
--- a/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
+++ b/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="Rd898866200114639"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R6f144dcca86f4f2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="Rc54e7f51d27346ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="Rb3317623790f4274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R4cbfed1ffbbc41e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="R19d9b030fedd4b1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="R67f3f16688f046d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R1723f3a68fd741f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="R65b22a1307f24117"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="R6f0a1e9d317f4263"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R35cef73e2235402c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="R9c357a8b5ee24f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="R636c527b03714035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R69e2490df172448d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="R68e0163e5a234174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="Rf9756e24bc154631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R0d35607cd0174b1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="R6b56ff7f83804398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neon Architecture" sheetId="11" r:id="R2f529141c0f04b73"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="AutomationOptions">Lists!$C$2:$C$4</x:definedName>
@@ -4466,7 +4467,7 @@
     <x:numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -4546,8 +4547,20 @@
       <x:color rgb="FF9A6700"/>
       <x:name val="Aptos Narrow"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF064E3B"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF166534"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -4619,8 +4632,18 @@
         <x:fgColor rgb="FFF3F8F9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD1FAE5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="13">
+  <x:borders count="22">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -4754,12 +4777,102 @@
         <x:color rgb="FFB6CDD1"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="76">
+  <x:cellXfs count="114">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -4960,6 +5073,94 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -9319,8 +9520,155 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4dcade8c7684f4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a080bbf51b94c56"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="77" t="str">
+        <x:v>Neon-Only Database Architecture — SQA</x:v>
+      </x:c>
+      <x:c r="B1" s="77"/>
+      <x:c r="C1" s="77"/>
+      <x:c r="D1" s="77"/>
+      <x:c r="E1" s="77"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="80" t="str">
+        <x:v>Area</x:v>
+      </x:c>
+      <x:c r="B3" s="80" t="str">
+        <x:v>Verification</x:v>
+      </x:c>
+      <x:c r="C3" s="80" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="D3" s="80" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="E3" s="80" t="str">
+        <x:v>Remaining limitation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A4" s="99" t="str">
+        <x:v>Runtime selection</x:v>
+      </x:c>
+      <x:c r="B4" s="100" t="str">
+        <x:v>Launcher accepts only the configured Neon staging URL</x:v>
+      </x:c>
+      <x:c r="C4" s="111" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D4" s="100" t="str">
+        <x:v>Windows startup and runtime-state verification</x:v>
+      </x:c>
+      <x:c r="E4" s="101" t="str">
+        <x:v>Internet and Neon service required</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="184.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A5" s="102" t="str">
+        <x:v>Local fallback removal</x:v>
+      </x:c>
+      <x:c r="B5" s="103" t="str">
+        <x:v>PostgreSQL Compose service, dump transfer, backup worker, device lock, and SQLite runtime switches removed</x:v>
+      </x:c>
+      <x:c r="C5" s="112" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D5" s="103" t="str">
+        <x:v>Repository and launcher inspection</x:v>
+      </x:c>
+      <x:c r="E5" s="104" t="str">
+        <x:v>Historical SQA reports remain labeled as superseded evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A6" s="102" t="str">
+        <x:v>Private package</x:v>
+      </x:c>
+      <x:c r="B6" s="103" t="str">
+        <x:v>Only .env, .gitignore, and README remain; account roster is tracked separately without passwords</x:v>
+      </x:c>
+      <x:c r="C6" s="112" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D6" s="103" t="str">
+        <x:v>verify-private-config.ps1 and backend password-rejection test</x:v>
+      </x:c>
+      <x:c r="E6" s="104" t="str">
+        <x:v>Secrets must be provisioned securely on each authorized computer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A7" s="102" t="str">
+        <x:v>Backend regression</x:v>
+      </x:c>
+      <x:c r="B7" s="103" t="str">
+        <x:v>179 backend tests and pip dependency check</x:v>
+      </x:c>
+      <x:c r="C7" s="112" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D7" s="103" t="str">
+        <x:v>Local automated gate on 2026-08-28</x:v>
+      </x:c>
+      <x:c r="E7" s="104" t="str">
+        <x:v>None observed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A8" s="102" t="str">
+        <x:v>Flutter regression</x:v>
+      </x:c>
+      <x:c r="B8" s="103" t="str">
+        <x:v>Static analysis, 51 tests, and release web build</x:v>
+      </x:c>
+      <x:c r="C8" s="112" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D8" s="103" t="str">
+        <x:v>Local automated gate on 2026-08-28</x:v>
+      </x:c>
+      <x:c r="E8" s="104" t="str">
+        <x:v>None observed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A9" s="105" t="str">
+        <x:v>Service health</x:v>
+      </x:c>
+      <x:c r="B9" s="106" t="str">
+        <x:v>Frontend, backend, sandbox, Alembic migration, and Neon selection</x:v>
+      </x:c>
+      <x:c r="C9" s="113" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D9" s="106" t="str">
+        <x:v>Local Windows runtime on ports 8180/5100/5101</x:v>
+      </x:c>
+      <x:c r="E9" s="107" t="str">
+        <x:v>Physical Ubuntu lab-computer smoke test not repeated</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -10441,11 +10789,11 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="R2563e8e0d55d45a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="Rc0d7d38dc9c045fc"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5d9394dcce34073"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f3066f4c26243ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21466,7 +21814,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ab06e18915a43de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2cbdad1db504148"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22142,7 +22490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fdc2898cde147fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22c83092c3214e1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40219,7 +40567,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94704f5617f44be9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bd032b84b3a41d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40304,7 +40652,7 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>182 tests passed; pip check and compileall passed.</x:v>
+        <x:v>179 tests passed with tracked-roster password protection; pip check and compileall passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38.099998474121094" customHeight="1">
@@ -41387,7 +41735,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5d0d278080c4411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9567927eb964575"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41612,7 +41960,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="61" t="str">
-        <x:v>Windows local staging verification | 2026-08-28 | Not committed or pushed</x:v>
+        <x:v>Windows local staging verification | 2026-08-28 | Implementation: staging main v5.3; final QA follow-up local</x:v>
       </x:c>
       <x:c r="B2" s="61"/>
       <x:c r="C2" s="61"/>
@@ -41837,19 +42185,19 @@
         <x:v>JSON</x:v>
       </x:c>
       <x:c r="C13" s="68" t="str">
-        <x:v>Private account importer</x:v>
+        <x:v>Tracked password-free account roster</x:v>
       </x:c>
       <x:c r="D13" s="68" t="str">
-        <x:v>File changes synchronize safely without deleting history</x:v>
+        <x:v>Every clone receives account metadata while passwords and hashes remain outside Git</x:v>
       </x:c>
       <x:c r="E13" s="72" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F13" s="68" t="str">
-        <x:v>Private JSON is read from local_handoff_package and temporary passwords are cleared after hashing.</x:v>
+        <x:v>backend/data/study_accounts.json contains metadata only; backend rejects temporary passwords in the canonical roster.</x:v>
       </x:c>
       <x:c r="G13" s="68" t="str">
-        <x:v>File is ignored by Git because it may contain credentials.</x:v>
+        <x:v>Create and reset passwords through Instructor Studio; hashes remain in Neon.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -41857,22 +42205,22 @@
         <x:v>V52-010</x:v>
       </x:c>
       <x:c r="B14" s="69" t="str">
-        <x:v>Fallback</x:v>
+        <x:v>Neon</x:v>
       </x:c>
       <x:c r="C14" s="69" t="str">
-        <x:v>Explicit local PostgreSQL mode</x:v>
+        <x:v>Neon-only database runtime</x:v>
       </x:c>
       <x:c r="D14" s="69" t="str">
-        <x:v>Offline mode remains usable</x:v>
+        <x:v>Startup requires the authorized Neon staging database; no local PostgreSQL, dump restore, backup worker, or device lock remains</x:v>
       </x:c>
       <x:c r="E14" s="73" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F14" s="69" t="str">
-        <x:v>Frontend/API/sandbox healthy; final verified dump created on stop.</x:v>
+        <x:v>Windows start/stop, private-config validation, Alembic migration, runtime-state, and service health checks passed. Internet and Neon availability are required.</x:v>
       </x:c>
       <x:c r="G14" s="69" t="str">
-        <x:v>Fallback snapshot does not continuously sync with Neon.</x:v>
+        <x:v>Requires internet access and Neon availability; no offline database mode remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -41892,7 +42240,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F15" s="68" t="str">
-        <x:v>182 tests; pip check clean; compileall clean.</x:v>
+        <x:v>179 tests after retiring obsolete database-transfer coverage and adding tracked-roster password protection; pip check clean; compileall clean.</x:v>
       </x:c>
       <x:c r="G15" s="68" t="str">
         <x:v>None observed.</x:v>

</xml_diff>

<commit_message>
v5.4: centralize local configuration
</commit_message>
<xml_diff>
--- a/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
+++ b/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="R6f0a1e9d317f4263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R35cef73e2235402c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="R9c357a8b5ee24f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="R636c527b03714035"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R69e2490df172448d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="R68e0163e5a234174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="Rf9756e24bc154631"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R0d35607cd0174b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="R6b56ff7f83804398"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neon Architecture" sheetId="11" r:id="R2f529141c0f04b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="R7a9d437e854c4318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R40bcb85935b84a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="R4abe26d0e0c947f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="R26658c0cd0544b70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="Refef22d409ad441a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="Rb9150a93d70b4bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="Rc02709079e754899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R2bad74f4a06d40ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="R4057fff2478f406e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neon Architecture" sheetId="11" r:id="Rb480ec69a1da4f72"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="AutomationOptions">Lists!$C$2:$C$4</x:definedName>
@@ -9520,7 +9520,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a080bbf51b94c56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8bceb7a9e944c26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9598,10 +9598,10 @@
     </x:row>
     <x:row r="6" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A6" s="102" t="str">
-        <x:v>Private package</x:v>
+        <x:v>Private configuration</x:v>
       </x:c>
       <x:c r="B6" s="103" t="str">
-        <x:v>Only .env, .gitignore, and README remain; account roster is tracked separately without passwords</x:v>
+        <x:v>One ignored repository-root .env; account roster is tracked separately without passwords</x:v>
       </x:c>
       <x:c r="C6" s="112" t="str">
         <x:v>PASS</x:v>
@@ -9610,7 +9610,7 @@
         <x:v>verify-private-config.ps1 and backend password-rejection test</x:v>
       </x:c>
       <x:c r="E6" s="104" t="str">
-        <x:v>Secrets must be provisioned securely on each authorized computer</x:v>
+        <x:v>The .env must be provisioned securely on each authorized computer</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -10789,11 +10789,11 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="Rc0d7d38dc9c045fc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="Rf4e5e8a433c64bc7"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f3066f4c26243ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra50390abfded4f27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21814,7 +21814,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2cbdad1db504148"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51e8131621184af3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22490,7 +22490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22c83092c3214e1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72f72d005c1d451e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40567,7 +40567,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bd032b84b3a41d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1a60ecea30c4e81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41735,7 +41735,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9567927eb964575"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0e41d7fdb6b4955"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
v5.5: repair assignment grading integrity
</commit_message>
<xml_diff>
--- a/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
+++ b/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="R7a9d437e854c4318"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R40bcb85935b84a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="R4abe26d0e0c947f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="R26658c0cd0544b70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="Refef22d409ad441a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="Rb9150a93d70b4bc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="Rc02709079e754899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R2bad74f4a06d40ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="R4057fff2478f406e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neon Architecture" sheetId="11" r:id="Rb480ec69a1da4f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="Ra02a1c6288b14acc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R398aef92e2d945ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="R487603662cae4e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="R1ab116dcfd8342ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R8223eab16efd48de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="Red87adc71b1c44e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="R4f624fae71b942db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R27c4837c5016469c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="Ra9b62b9afae647ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neon Architecture" sheetId="11" r:id="R8c702606027f4621"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grading Integrity QA" sheetId="12" r:id="Ra42f14a5809a4c32"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="AutomationOptions">Lists!$C$2:$C$4</x:definedName>
@@ -4467,7 +4468,7 @@
     <x:numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="16">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -4559,8 +4560,37 @@
       <x:color rgb="FF166534"/>
       <x:name val="Aptos Narrow"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF2F5D31"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -4642,8 +4672,68 @@
         <x:fgColor rgb="FFD1FAE5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F6B78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F6B78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F6B78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="22">
+  <x:borders count="24">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -4867,12 +4957,25 @@
         <x:color rgb="FFD1D5DB"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C6D1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFB8C6D1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C6D1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="114">
+  <x:cellXfs count="157">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -5162,6 +5265,97 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="16" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="20" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="16" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="23" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="20" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="24" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="24" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="24" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="16" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="27" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="27" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="28" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="28" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="28" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -9520,7 +9714,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8bceb7a9e944c26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8145fec198144cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9668,6 +9862,333 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
   </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="148" t="str">
+        <x:v>Assignment grading integrity repair</x:v>
+      </x:c>
+      <x:c r="B1" s="148"/>
+      <x:c r="C1" s="148"/>
+      <x:c r="D1" s="148"/>
+      <x:c r="E1" s="148"/>
+      <x:c r="F1" s="148"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="149" t="str">
+        <x:v>Test date</x:v>
+      </x:c>
+      <x:c r="B2" s="150" t="n">
+        <x:v>46288.791666666664</x:v>
+      </x:c>
+      <x:c r="C2" s="149" t="str">
+        <x:v>Branch</x:v>
+      </x:c>
+      <x:c r="D2" s="151" t="str">
+        <x:v>fix/grading-integrity</x:v>
+      </x:c>
+      <x:c r="E2" s="149" t="str">
+        <x:v>Release state</x:v>
+      </x:c>
+      <x:c r="F2" s="151" t="str">
+        <x:v>Local only; not committed or pushed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="149" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="B3" s="151" t="str">
+        <x:v>Assignments 1-6 grading, scoring, feedback, instructor validation, Flutter compatibility, and real ROS 2 execution</x:v>
+      </x:c>
+      <x:c r="C3" s="151"/>
+      <x:c r="D3" s="151"/>
+      <x:c r="E3" s="151"/>
+      <x:c r="F3" s="151"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="114"/>
+      <x:c r="B4" s="114"/>
+      <x:c r="C4" s="114"/>
+      <x:c r="D4" s="114"/>
+      <x:c r="E4" s="114"/>
+      <x:c r="F4" s="114"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="153" t="str">
+        <x:v>Check ID</x:v>
+      </x:c>
+      <x:c r="B5" s="153" t="str">
+        <x:v>Area</x:v>
+      </x:c>
+      <x:c r="C5" s="153" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="D5" s="153" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="E5" s="153" t="str">
+        <x:v>Issue repaired</x:v>
+      </x:c>
+      <x:c r="F5" s="153" t="str">
+        <x:v>Remaining limitation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="129" t="str">
+        <x:v>GI-001</x:v>
+      </x:c>
+      <x:c r="B6" s="129" t="str">
+        <x:v>Run endpoint</x:v>
+      </x:c>
+      <x:c r="C6" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D6" s="129" t="str">
+        <x:v>Run and Submit now use the same assignment grader.</x:v>
+      </x:c>
+      <x:c r="E6" s="129" t="str">
+        <x:v>Executable code can no longer receive an automatic 100% Run result.</x:v>
+      </x:c>
+      <x:c r="F6" s="129" t="str">
+        <x:v>None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="129" t="str">
+        <x:v>GI-002</x:v>
+      </x:c>
+      <x:c r="B7" s="129" t="str">
+        <x:v>Assignment 1</x:v>
+      </x:c>
+      <x:c r="C7" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D7" s="129" t="str">
+        <x:v>Official 100%; mixed 25%; displayed constants rejected.</x:v>
+      </x:c>
+      <x:c r="E7" s="129" t="str">
+        <x:v>Grades a reusable Bug2 function across hidden coordinate scenarios.</x:v>
+      </x:c>
+      <x:c r="F7" s="129" t="str">
+        <x:v>Hidden cases remain server-only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="129" t="str">
+        <x:v>GI-003</x:v>
+      </x:c>
+      <x:c r="B8" s="129" t="str">
+        <x:v>Assignment 2</x:v>
+      </x:c>
+      <x:c r="C8" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D8" s="129" t="str">
+        <x:v>Official 100%; mixed 25%; displayed constants rejected.</x:v>
+      </x:c>
+      <x:c r="E8" s="129" t="str">
+        <x:v>Grades a reusable Bug route function across hidden coordinate scenarios.</x:v>
+      </x:c>
+      <x:c r="F8" s="129" t="str">
+        <x:v>Hidden cases remain server-only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="129" t="str">
+        <x:v>GI-004</x:v>
+      </x:c>
+      <x:c r="B9" s="129" t="str">
+        <x:v>Assignment 3</x:v>
+      </x:c>
+      <x:c r="C9" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D9" s="129" t="str">
+        <x:v>Official 100%; mixed 50%; displayed constants rejected.</x:v>
+      </x:c>
+      <x:c r="E9" s="129" t="str">
+        <x:v>Grades all eight route outputs across cases where either elevator can win.</x:v>
+      </x:c>
+      <x:c r="F9" s="129" t="str">
+        <x:v>Eight 12.5% checks display as a rounded whole percentage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="129" t="str">
+        <x:v>GI-005</x:v>
+      </x:c>
+      <x:c r="B10" s="129" t="str">
+        <x:v>Assignment 4</x:v>
+      </x:c>
+      <x:c r="C10" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D10" s="129" t="str">
+        <x:v>Official 100%; mixed 60%; displayed constants rejected.</x:v>
+      </x:c>
+      <x:c r="E10" s="129" t="str">
+        <x:v>Expanded grading from two 50% checks to five 20% checks.</x:v>
+      </x:c>
+      <x:c r="F10" s="129" t="str">
+        <x:v>None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="129" t="str">
+        <x:v>GI-006</x:v>
+      </x:c>
+      <x:c r="B11" s="129" t="str">
+        <x:v>Assignment 5 ROS 2</x:v>
+      </x:c>
+      <x:c r="C11" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D11" s="129" t="str">
+        <x:v>Real Docker ROS grader passed 7 of 7 checks.</x:v>
+      </x:c>
+      <x:c r="E11" s="129" t="str">
+        <x:v>Rubric weights now match the behavior-harness weights.</x:v>
+      </x:c>
+      <x:c r="F11" s="129" t="str">
+        <x:v>Docker Desktop Linux containers are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="129" t="str">
+        <x:v>GI-007</x:v>
+      </x:c>
+      <x:c r="B12" s="129" t="str">
+        <x:v>Assignment 6 ROS 2</x:v>
+      </x:c>
+      <x:c r="C12" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D12" s="129" t="str">
+        <x:v>Real Docker ROS grader passed 9 of 9 checks.</x:v>
+      </x:c>
+      <x:c r="E12" s="129" t="str">
+        <x:v>Rubric weights now match the behavior-harness weights.</x:v>
+      </x:c>
+      <x:c r="F12" s="129" t="str">
+        <x:v>Docker Desktop Linux containers are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="129" t="str">
+        <x:v>GI-008</x:v>
+      </x:c>
+      <x:c r="B13" s="129" t="str">
+        <x:v>Instructor validation</x:v>
+      </x:c>
+      <x:c r="C13" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D13" s="129" t="str">
+        <x:v>Function-grader assignments validate, edit, and publish in automated tests.</x:v>
+      </x:c>
+      <x:c r="E13" s="129" t="str">
+        <x:v>Assignment Studio recognizes and validates the new grader configuration.</x:v>
+      </x:c>
+      <x:c r="F13" s="129" t="str">
+        <x:v>None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="129" t="str">
+        <x:v>GI-009</x:v>
+      </x:c>
+      <x:c r="B14" s="129" t="str">
+        <x:v>Backend regression</x:v>
+      </x:c>
+      <x:c r="C14" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D14" s="129" t="str">
+        <x:v>Final backend regression gate passed all 200 tests.</x:v>
+      </x:c>
+      <x:c r="E14" s="129" t="str">
+        <x:v>No backend regression detected.</x:v>
+      </x:c>
+      <x:c r="F14" s="129" t="str">
+        <x:v>None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="129" t="str">
+        <x:v>GI-010</x:v>
+      </x:c>
+      <x:c r="B15" s="129" t="str">
+        <x:v>Python dependencies</x:v>
+      </x:c>
+      <x:c r="C15" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D15" s="129" t="str">
+        <x:v>pip check reported no broken requirements.</x:v>
+      </x:c>
+      <x:c r="E15" s="129" t="str">
+        <x:v>No dependency conflict detected.</x:v>
+      </x:c>
+      <x:c r="F15" s="129" t="str">
+        <x:v>None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="129" t="str">
+        <x:v>GI-011</x:v>
+      </x:c>
+      <x:c r="B16" s="129" t="str">
+        <x:v>Flutter client</x:v>
+      </x:c>
+      <x:c r="C16" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D16" s="129" t="str">
+        <x:v>Static analysis passed; 52 tests passed; release web build completed.</x:v>
+      </x:c>
+      <x:c r="E16" s="129" t="str">
+        <x:v>Updated assignment criteria and instructions remain client-compatible.</x:v>
+      </x:c>
+      <x:c r="F16" s="129" t="str">
+        <x:v>No physical mobile-device test was required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="129" t="str">
+        <x:v>GI-012</x:v>
+      </x:c>
+      <x:c r="B17" s="129" t="str">
+        <x:v>Repository state</x:v>
+      </x:c>
+      <x:c r="C17" s="156" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D17" s="129" t="str">
+        <x:v>Changes are isolated on fix/grading-integrity.</x:v>
+      </x:c>
+      <x:c r="E17" s="129" t="str">
+        <x:v>Production and remote main were not modified.</x:v>
+      </x:c>
+      <x:c r="F17" s="129" t="str">
+        <x:v>Commit and push require separate approval.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -10789,11 +11310,11 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="Rf4e5e8a433c64bc7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="Rd54f9bf16d014c0e"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra50390abfded4f27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R381ae7327f2149e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21814,7 +22335,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51e8131621184af3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fa80bd2e90f4066"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22490,7 +23011,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72f72d005c1d451e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b651e71370a4482"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40567,7 +41088,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1a60ecea30c4e81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50e9f3e9e6184ba1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41735,7 +42256,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0e41d7fdb6b4955"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9f27b413aab4d4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
v5.5: fix stale grading results and weighted scores
</commit_message>
<xml_diff>
--- a/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
+++ b/docs/sqa/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="Ra02a1c6288b14acc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R398aef92e2d945ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="R487603662cae4e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="R1ab116dcfd8342ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R8223eab16efd48de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="Red87adc71b1c44e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="R4f624fae71b942db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R27c4837c5016469c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="Ra9b62b9afae647ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neon Architecture" sheetId="11" r:id="R8c702606027f4621"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grading Integrity QA" sheetId="12" r:id="Ra42f14a5809a4c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4 SQA Report" sheetId="9" r:id="Rd158b9fa5f4c4208"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="7" r:id="R723135846bbf4e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="6" r:id="Rc2b411fcc97740f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Matrix" sheetId="5" r:id="Rfb5dadab684d4184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R4df60db466ae4fbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Sign-off" sheetId="3" r:id="R5e25eae9ca994776"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runbook" sheetId="2" r:id="R46f9b4bf12b9417c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="Ra82007c8245f4e19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5.2 Neon &amp; Accounts" sheetId="10" r:id="R601f0b0dd9204a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neon Architecture" sheetId="11" r:id="R75b060f5c3c14e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grading Integrity QA" sheetId="12" r:id="Re31f81f2bb56465b"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="AutomationOptions">Lists!$C$2:$C$4</x:definedName>
@@ -4975,7 +4975,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="157">
+  <x:cellXfs count="158">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -5356,6 +5356,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="19" fillId="28" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -9714,7 +9717,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8145fec198144cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf25ac87975034ed3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10186,6 +10189,86 @@
       </x:c>
       <x:c r="F17" s="129" t="str">
         <x:v>Commit and push require separate approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="52" hidden="0" customHeight="1">
+      <x:c r="A18" s="157" t="str">
+        <x:v>GI-013</x:v>
+      </x:c>
+      <x:c r="B18" s="157" t="str">
+        <x:v>Student mutation matrix</x:v>
+      </x:c>
+      <x:c r="C18" s="157" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D18" s="157" t="str">
+        <x:v>Assignments 1-4 missing/renamed helpers: 0%; Assignment 5 missing publisher: 20%; Assignment 6 missing publisher: 10%</x:v>
+      </x:c>
+      <x:c r="E18" s="157" t="str">
+        <x:v>Broken or incomplete submissions no longer appear to earn a false 100% score</x:v>
+      </x:c>
+      <x:c r="F18" s="157" t="str">
+        <x:v>ROS partial-credit weights are intentional and remain server-authoritative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="52" hidden="0" customHeight="1">
+      <x:c r="A19" s="157" t="str">
+        <x:v>GI-014</x:v>
+      </x:c>
+      <x:c r="B19" s="157" t="str">
+        <x:v>Edited-code result state</x:v>
+      </x:c>
+      <x:c r="C19" s="157" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D19" s="157" t="str">
+        <x:v>Manual browser QA: correct answer 100%, edit code, stale Results panel hides and header labels the value as Previous score</x:v>
+      </x:c>
+      <x:c r="E19" s="157" t="str">
+        <x:v>A previous successful result can no longer be mistaken for the edited, untested code</x:v>
+      </x:c>
+      <x:c r="F19" s="157" t="str">
+        <x:v>Completed remains a historical achievement after a prior successful attempt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52" hidden="0" customHeight="1">
+      <x:c r="A20" s="157" t="str">
+        <x:v>GI-015</x:v>
+      </x:c>
+      <x:c r="B20" s="157" t="str">
+        <x:v>Weighted score display</x:v>
+      </x:c>
+      <x:c r="C20" s="157" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D20" s="157" t="str">
+        <x:v>UI uses backend score; check pass rate is displayed separately. Regression test covers 35% score with 1/2 checks</x:v>
+      </x:c>
+      <x:c r="E20" s="157" t="str">
+        <x:v>Frontend no longer replaces assignment-specific weights with an unweighted check fraction</x:v>
+      </x:c>
+      <x:c r="F20" s="157" t="str">
+        <x:v>None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="52" hidden="0" customHeight="1">
+      <x:c r="A21" s="157" t="str">
+        <x:v>GI-016</x:v>
+      </x:c>
+      <x:c r="B21" s="157" t="str">
+        <x:v>Frontend regression</x:v>
+      </x:c>
+      <x:c r="C21" s="157" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D21" s="157" t="str">
+        <x:v>Flutter analyze passed; 52 tests passed; release web build passed; narrow-screen feedback test passed</x:v>
+      </x:c>
+      <x:c r="E21" s="157" t="str">
+        <x:v>Student-facing score and stale-result changes were regression checked</x:v>
+      </x:c>
+      <x:c r="F21" s="157" t="str">
+        <x:v>No physical mobile-device test was performed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11310,11 +11393,11 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="Rd54f9bf16d014c0e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="R3055a45e8b4e4c7d"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R381ae7327f2149e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdc4cb549a56455c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22335,7 +22418,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fa80bd2e90f4066"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fbfeba095114089"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23011,7 +23094,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b651e71370a4482"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd51d5116cdd84f1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41088,7 +41171,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50e9f3e9e6184ba1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa49dd4e24f14d99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42256,7 +42339,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9f27b413aab4d4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ce2012cadbb4865"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>